<commit_message>
1.0.6 release. Updates for email subject lines
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\55651C\Documents\GitHub\P002_090_PayCyleAfternoon_Dispatcher\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\57841C\Documents\UiPath\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{977E1869-97A5-40F6-954D-7428BAC06BA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABF3CEC1-98C4-4B64-A8B9-DC61FD47D28A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -193,9 +193,6 @@
     <t>EmailSubject</t>
   </si>
   <si>
-    <t>Bot Completed</t>
-  </si>
-  <si>
     <t>Success Email Subject</t>
   </si>
   <si>
@@ -997,10 +994,6 @@
     <t>SE_3CCEmailAddress</t>
   </si>
   <si>
-    <t xml:space="preserve">Hello Team,&lt;br&gt;&lt;br&gt;This email notification was raised for P002_090_PayCycleAfternoon process
- &lt;br&gt;The process executed successfully and Paycycle data was added to the queue. In case of any issues with the automation, please reach out to the RPA Support Team.&lt;br&gt;&lt;br&gt;  Thanks,&lt;br&gt;Automation Team  </t>
-  </si>
-  <si>
     <t>\d+\s-\s\w+\sno success</t>
   </si>
   <si>
@@ -1218,6 +1211,12 @@
   </si>
   <si>
     <t>ProcessRunFolderName</t>
+  </si>
+  <si>
+    <t>Hello Team,&lt;br&gt;&lt;br&gt; OKBATCNN job was successfully verified and all the 3 pay cycles have been added to bot queue for processing.&lt;br&gt;Note: This email is generated by the system. Please refrain from replying directly to this email. For assistance, please contact the RPA support team at acoesupport@omes.ok.gov&lt;br&gt;&lt;br&gt;Thanks,&lt;br&gt;Pay Cycle Afternoon Automation</t>
+  </si>
+  <si>
+    <t>OKBATCNN Job Validation and Addition of 3 Pay Cycles for Processing {Date}</t>
   </si>
   <si>
     <t>PROD</t>
@@ -1578,9 +1577,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1618,7 +1617,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1724,7 +1723,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1866,7 +1865,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1919,10 +1918,10 @@
     </row>
     <row r="2" spans="1:26">
       <c r="A2" s="2" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>20</v>
@@ -1945,7 +1944,7 @@
         <v>19</v>
       </c>
       <c r="B4" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>21</v>
@@ -1956,7 +1955,7 @@
         <v>42</v>
       </c>
       <c r="B5" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C5" t="s">
         <v>43</v>
@@ -1964,7 +1963,7 @@
     </row>
     <row r="6" spans="1:26">
       <c r="A6" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="B6" t="str">
         <f>_xlfn.CONCAT(Constants!$B$18,"/P002_090_PayCycleAfternoon")</f>
@@ -1976,7 +1975,7 @@
         <v>48</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>319</v>
+        <v>391</v>
       </c>
       <c r="C7" t="s">
         <v>49</v>
@@ -1987,182 +1986,182 @@
         <v>50</v>
       </c>
       <c r="B8" t="s">
+        <v>392</v>
+      </c>
+      <c r="C8" t="s">
         <v>51</v>
-      </c>
-      <c r="C8" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="9" spans="1:26" ht="43.5">
       <c r="A9" t="s">
+        <v>52</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="C9" t="s">
         <v>53</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="C9" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="10" spans="1:26">
       <c r="A10" t="s">
+        <v>54</v>
+      </c>
+      <c r="B10" t="s">
         <v>55</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
         <v>56</v>
-      </c>
-      <c r="C10" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="11" spans="1:26">
       <c r="A11" t="s">
+        <v>57</v>
+      </c>
+      <c r="B11" t="s">
         <v>58</v>
       </c>
-      <c r="B11" t="s">
+      <c r="C11" t="s">
         <v>59</v>
-      </c>
-      <c r="C11" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="12" spans="1:26">
       <c r="A12" t="s">
+        <v>60</v>
+      </c>
+      <c r="B12" t="s">
         <v>61</v>
       </c>
-      <c r="B12" t="s">
+      <c r="C12" t="s">
         <v>62</v>
-      </c>
-      <c r="C12" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="13" spans="1:26">
       <c r="A13" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B13" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C13" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="14" spans="1:26">
       <c r="A14" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="B14" s="21" t="s">
+        <v>368</v>
+      </c>
+      <c r="C14" s="5" t="s">
         <v>65</v>
-      </c>
-      <c r="B14" s="21" t="s">
-        <v>370</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="15" spans="1:26">
       <c r="A15" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="B15" s="21" t="s">
+        <v>369</v>
+      </c>
+      <c r="C15" s="5" t="s">
         <v>67</v>
-      </c>
-      <c r="B15" s="21" t="s">
-        <v>371</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="16" spans="1:26">
       <c r="A16" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="B16" s="22" t="s">
+        <v>370</v>
+      </c>
+      <c r="C16" s="5" t="s">
         <v>69</v>
-      </c>
-      <c r="B16" s="22" t="s">
-        <v>372</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" s="5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B17">
         <v>5000</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B18">
         <v>5</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B19">
         <v>2</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" s="23" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B20" t="b">
         <v>1</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B21">
         <v>20</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B22" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="B23" t="s">
         <v>85</v>
-      </c>
-      <c r="B23" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="B24" t="s">
         <v>88</v>
-      </c>
-      <c r="B24" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" s="20" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B25">
         <v>50</v>
@@ -2170,15 +2169,15 @@
     </row>
     <row r="26" spans="1:3">
       <c r="A26" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="B26" t="s">
         <v>91</v>
-      </c>
-      <c r="B26" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="27" spans="1:3">
       <c r="A27" s="17" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B27">
         <v>10</v>
@@ -2186,7 +2185,7 @@
     </row>
     <row r="28" spans="1:3">
       <c r="A28" s="7" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B28">
         <v>1</v>
@@ -2194,63 +2193,63 @@
     </row>
     <row r="29" spans="1:3">
       <c r="A29" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="B29" t="s">
         <v>125</v>
-      </c>
-      <c r="B29" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="30" spans="1:3">
       <c r="A30" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="B30" t="s">
         <v>127</v>
-      </c>
-      <c r="B30" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="31" spans="1:3">
       <c r="A31" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="B31" t="s">
         <v>129</v>
-      </c>
-      <c r="B31" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="32" spans="1:3">
       <c r="A32" s="7" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B32" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="33" spans="1:2">
       <c r="A33" s="8" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B33" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
     </row>
     <row r="34" spans="1:2">
       <c r="A34" s="10" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B34" s="11" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
     </row>
     <row r="35" spans="1:2">
       <c r="A35" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B35" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="36" spans="1:2">
       <c r="A36" s="10" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B36">
         <v>5</v>
@@ -2258,15 +2257,15 @@
     </row>
     <row r="37" spans="1:2">
       <c r="A37" s="19" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B37" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="38" spans="1:2">
       <c r="A38" s="18" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B38" t="b">
         <v>1</v>
@@ -2274,31 +2273,31 @@
     </row>
     <row r="39" spans="1:2">
       <c r="A39" s="13" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B39" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
     </row>
     <row r="40" spans="1:2">
       <c r="A40" s="12" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B40" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="41" spans="1:2" ht="58">
       <c r="A41" s="12" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="42" spans="1:2">
       <c r="A42" s="13" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B42" s="3">
         <v>15</v>
@@ -2306,151 +2305,151 @@
     </row>
     <row r="43" spans="1:2">
       <c r="A43" s="16" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B43" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="44" spans="1:2" ht="43.5">
       <c r="A44" s="12" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="45" spans="1:2">
       <c r="A45" s="19" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B45" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="46" spans="1:2" ht="29">
       <c r="A46" s="19" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="47" spans="1:2">
       <c r="A47" s="19" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="B47" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="48" spans="1:2" ht="58">
       <c r="A48" s="19" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="49" spans="1:2">
       <c r="A49" s="12" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B49" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="50" spans="1:2" ht="29">
       <c r="A50" s="12" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="51" spans="1:2">
       <c r="A51" s="19" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="B51" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="52" spans="1:2" ht="43.5">
       <c r="A52" s="19" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="53" spans="1:2">
       <c r="A53" s="24" t="s">
+        <v>382</v>
+      </c>
+      <c r="B53" t="s">
         <v>384</v>
-      </c>
-      <c r="B53" t="s">
-        <v>386</v>
       </c>
     </row>
     <row r="54" spans="1:2" ht="43.5">
       <c r="A54" s="24" t="s">
+        <v>383</v>
+      </c>
+      <c r="B54" s="3" t="s">
         <v>385</v>
-      </c>
-      <c r="B54" s="3" t="s">
-        <v>387</v>
       </c>
     </row>
     <row r="55" spans="1:2">
       <c r="A55" s="15" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B55" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="56" spans="1:2">
       <c r="A56" s="14" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="B56" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="57" spans="1:2">
       <c r="A57" s="14" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B57" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="58" spans="1:2">
       <c r="A58" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B58" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="59" spans="1:2">
       <c r="A59" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B59" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="60" spans="1:2">
       <c r="A60" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B60" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="61" spans="1:2">
       <c r="A61" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B61" s="2" t="str">
         <f>Constants!$B$18</f>
@@ -2459,7 +2458,7 @@
     </row>
     <row r="62" spans="1:2">
       <c r="A62" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="B62" t="b">
         <v>1</v>
@@ -2467,12 +2466,12 @@
     </row>
     <row r="63" spans="1:2">
       <c r="A63" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="64" spans="1:2">
       <c r="A64" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B64">
         <v>2</v>
@@ -2480,15 +2479,15 @@
     </row>
     <row r="65" spans="1:2">
       <c r="A65" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="66" spans="1:2">
       <c r="A66" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="B66" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
     </row>
   </sheetData>
@@ -2677,7 +2676,7 @@
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="B18" t="s">
         <v>393</v>
@@ -2705,7 +2704,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>27</v>
@@ -2738,17 +2737,17 @@
     </row>
     <row r="2" spans="1:26">
       <c r="A2" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C2" t="str">
         <f>_xlfn.CONCAT(Constants!$B$18,"/P002_090_PayCycleAfternoon")</f>
         <v>PROD/P002_090_PayCycleAfternoon</v>
       </c>
       <c r="D2" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
     </row>
     <row r="3" spans="1:26">
@@ -2756,7 +2755,7 @@
         <v>41</v>
       </c>
       <c r="B3" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="C3" t="str">
         <f>_xlfn.CONCAT(Constants!$B$18,"/P002_090_PayCycleAfternoon")</f>
@@ -2765,10 +2764,10 @@
     </row>
     <row r="4" spans="1:26">
       <c r="A4" t="s">
+        <v>321</v>
+      </c>
+      <c r="B4" t="s">
         <v>323</v>
-      </c>
-      <c r="B4" t="s">
-        <v>325</v>
       </c>
       <c r="C4" t="str">
         <f>_xlfn.CONCAT(Constants!$B$18,"/P002_090_PayCycleAfternoon")</f>
@@ -2780,7 +2779,7 @@
         <v>44</v>
       </c>
       <c r="B5" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="C5" t="str">
         <f>_xlfn.CONCAT(Constants!$B$18,"/P002_090_PayCycleAfternoon")</f>
@@ -2792,7 +2791,7 @@
         <v>45</v>
       </c>
       <c r="B6" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="C6" t="str">
         <f>_xlfn.CONCAT(Constants!$B$18,"/P002_090_PayCycleAfternoon")</f>
@@ -2804,7 +2803,7 @@
         <v>46</v>
       </c>
       <c r="B7" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="C7" t="str">
         <f>_xlfn.CONCAT(Constants!$B$18,"/P002_090_PayCycleAfternoon")</f>
@@ -2816,7 +2815,7 @@
         <v>47</v>
       </c>
       <c r="B8" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="C8" t="str">
         <f>_xlfn.CONCAT(Constants!$B$18,"/P002_090_PayCycleAfternoon")</f>
@@ -2825,10 +2824,10 @@
     </row>
     <row r="9" spans="1:26">
       <c r="A9" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B9" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="C9" t="str">
         <f>_xlfn.CONCAT(Constants!$B$18,"/P002_090_PayCycleAfternoon")</f>
@@ -2837,10 +2836,10 @@
     </row>
     <row r="10" spans="1:26">
       <c r="A10" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B10" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="C10" t="str">
         <f>_xlfn.CONCAT(Constants!$B$18,"/P002_090_PayCycleAfternoon")</f>
@@ -2849,10 +2848,10 @@
     </row>
     <row r="11" spans="1:26">
       <c r="A11" s="19" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B11" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="C11" t="str">
         <f>_xlfn.CONCAT(Constants!$B$18,"/P002_090_PayCycleAfternoon")</f>
@@ -2861,10 +2860,10 @@
     </row>
     <row r="12" spans="1:26">
       <c r="A12" s="19" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B12" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="C12" t="str">
         <f>_xlfn.CONCAT(Constants!$B$18,"/P002_090_PayCycleAfternoon")</f>
@@ -2873,10 +2872,10 @@
     </row>
     <row r="13" spans="1:26">
       <c r="A13" s="19" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B13" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="C13" t="str">
         <f>_xlfn.CONCAT(Constants!$B$18,"/P002_090_PayCycleAfternoon")</f>
@@ -2885,10 +2884,10 @@
     </row>
     <row r="14" spans="1:26">
       <c r="A14" s="19" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B14" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="C14" t="str">
         <f>_xlfn.CONCAT(Constants!$B$18,"/P002_090_PayCycleAfternoon")</f>
@@ -2897,10 +2896,10 @@
     </row>
     <row r="15" spans="1:26">
       <c r="A15" s="19" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B15" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="C15" t="str">
         <f>_xlfn.CONCAT(Constants!$B$18,"/P002_090_PayCycleAfternoon")</f>
@@ -2909,10 +2908,10 @@
     </row>
     <row r="16" spans="1:26">
       <c r="A16" s="19" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B16" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="C16" t="str">
         <f>_xlfn.CONCAT(Constants!$B$18,"/P002_090_PayCycleAfternoon")</f>
@@ -2921,10 +2920,10 @@
     </row>
     <row r="17" spans="1:3">
       <c r="A17" s="19" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B17" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="C17" t="str">
         <f>_xlfn.CONCAT(Constants!$B$18,"/P002_090_PayCycleAfternoon")</f>
@@ -2933,10 +2932,10 @@
     </row>
     <row r="18" spans="1:3">
       <c r="A18" s="19" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B18" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="C18" t="str">
         <f>_xlfn.CONCAT(Constants!$B$18,"/P002_090_PayCycleAfternoon")</f>
@@ -2945,10 +2944,10 @@
     </row>
     <row r="19" spans="1:3">
       <c r="A19" s="19" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="B19" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="C19" t="str">
         <f>_xlfn.CONCAT(Constants!$B$18,"/P002_090_PayCycleAfternoon")</f>
@@ -2957,10 +2956,10 @@
     </row>
     <row r="20" spans="1:3">
       <c r="A20" s="19" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="B20" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="C20" t="str">
         <f>_xlfn.CONCAT(Constants!$B$18,"/P002_090_PayCycleAfternoon")</f>
@@ -2969,10 +2968,10 @@
     </row>
     <row r="21" spans="1:3">
       <c r="A21" s="19" t="s">
+        <v>342</v>
+      </c>
+      <c r="B21" t="s">
         <v>344</v>
-      </c>
-      <c r="B21" t="s">
-        <v>346</v>
       </c>
       <c r="C21" t="str">
         <f>_xlfn.CONCAT(Constants!$B$18,"/P002_090_PayCycleAfternoon")</f>
@@ -2981,10 +2980,10 @@
     </row>
     <row r="22" spans="1:3">
       <c r="A22" s="19" t="s">
+        <v>343</v>
+      </c>
+      <c r="B22" t="s">
         <v>345</v>
-      </c>
-      <c r="B22" t="s">
-        <v>347</v>
       </c>
       <c r="C22" t="str">
         <f>_xlfn.CONCAT(Constants!$B$18,"/P002_090_PayCycleAfternoon")</f>
@@ -2993,10 +2992,10 @@
     </row>
     <row r="23" spans="1:3">
       <c r="A23" s="24" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="B23" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="C23" t="str">
         <f>_xlfn.CONCAT(Constants!$B$18,"/P002_090_PayCycleAfternoon")</f>
@@ -3005,10 +3004,10 @@
     </row>
     <row r="24" spans="1:3">
       <c r="A24" s="24" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="B24" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="C24" t="str">
         <f>_xlfn.CONCAT(Constants!$B$18,"/P002_090_PayCycleAfternoon")</f>
@@ -3017,10 +3016,10 @@
     </row>
     <row r="25" spans="1:3">
       <c r="A25" s="19" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="B25" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="C25" t="str">
         <f>_xlfn.CONCAT(Constants!$B$18,"/P002_090_PayCycleAfternoon")</f>
@@ -3079,722 +3078,722 @@
     </row>
     <row r="2" spans="1:26">
       <c r="A2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B2" t="s">
         <v>93</v>
-      </c>
-      <c r="B2" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="3" spans="1:26">
       <c r="A3" t="s">
+        <v>281</v>
+      </c>
+      <c r="B3" t="s">
         <v>282</v>
-      </c>
-      <c r="B3" t="s">
-        <v>283</v>
       </c>
     </row>
     <row r="4" spans="1:26">
       <c r="A4" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B4" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="5" spans="1:26">
       <c r="A5" t="s">
+        <v>94</v>
+      </c>
+      <c r="B5" t="s">
         <v>95</v>
-      </c>
-      <c r="B5" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="6" spans="1:26">
       <c r="A6" t="s">
+        <v>96</v>
+      </c>
+      <c r="B6" t="s">
         <v>97</v>
-      </c>
-      <c r="B6" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="7" spans="1:26">
       <c r="A7" t="s">
+        <v>98</v>
+      </c>
+      <c r="B7" t="s">
         <v>99</v>
-      </c>
-      <c r="B7" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="8" spans="1:26">
       <c r="A8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B8" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="9" spans="1:26">
       <c r="A9" t="s">
+        <v>105</v>
+      </c>
+      <c r="B9" t="s">
         <v>106</v>
-      </c>
-      <c r="B9" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="10" spans="1:26">
       <c r="A10" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="B10" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="11" spans="1:26">
       <c r="A11" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="B11" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
     </row>
     <row r="12" spans="1:26">
       <c r="A12" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="B12" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="13" spans="1:26">
       <c r="A13" t="s">
+        <v>297</v>
+      </c>
+      <c r="B13" t="s">
         <v>298</v>
-      </c>
-      <c r="B13" t="s">
-        <v>299</v>
       </c>
     </row>
     <row r="14" spans="1:26">
       <c r="A14" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="B14" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
     </row>
     <row r="15" spans="1:26">
       <c r="A15" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="B15" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
     </row>
     <row r="16" spans="1:26">
       <c r="A16" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="B16" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B17" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B18" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B19" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="B20" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B21" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="22" spans="1:2">
       <c r="A22" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B22" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="23" spans="1:2">
       <c r="A23" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B23" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="24" spans="1:2">
       <c r="A24" t="s">
+        <v>302</v>
+      </c>
+      <c r="B24" t="s">
         <v>303</v>
-      </c>
-      <c r="B24" t="s">
-        <v>304</v>
       </c>
     </row>
     <row r="25" spans="1:2">
       <c r="A25" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B25" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="26" spans="1:2">
       <c r="A26" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B26" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="27" spans="1:2">
       <c r="A27" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B27" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="28" spans="1:2">
       <c r="A28" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B28" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="29" spans="1:2">
       <c r="A29" t="s">
+        <v>247</v>
+      </c>
+      <c r="B29" t="s">
         <v>248</v>
-      </c>
-      <c r="B29" t="s">
-        <v>249</v>
       </c>
     </row>
     <row r="30" spans="1:2">
       <c r="A30" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B30" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="31" spans="1:2">
       <c r="A31" t="s">
+        <v>292</v>
+      </c>
+      <c r="B31" t="s">
         <v>293</v>
-      </c>
-      <c r="B31" t="s">
-        <v>294</v>
       </c>
     </row>
     <row r="32" spans="1:2">
       <c r="A32" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B32" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="33" spans="1:2">
       <c r="A33" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="B33" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
     </row>
     <row r="34" spans="1:2">
       <c r="A34" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="B34" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
     </row>
     <row r="35" spans="1:2">
       <c r="A35" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="B35" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
     </row>
     <row r="36" spans="1:2">
       <c r="A36" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B36" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="37" spans="1:2">
       <c r="A37" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B37" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="38" spans="1:2">
       <c r="A38" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B38" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="39" spans="1:2">
       <c r="A39" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B39" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="40" spans="1:2">
       <c r="A40" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B40" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="41" spans="1:2">
       <c r="A41" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B41" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="42" spans="1:2">
       <c r="A42" t="s">
+        <v>149</v>
+      </c>
+      <c r="B42" t="s">
         <v>150</v>
-      </c>
-      <c r="B42" t="s">
-        <v>151</v>
       </c>
     </row>
     <row r="43" spans="1:2">
       <c r="A43" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B43" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="44" spans="1:2">
       <c r="A44" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B44" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="45" spans="1:2">
       <c r="A45" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B45" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="46" spans="1:2">
       <c r="A46" t="s">
+        <v>289</v>
+      </c>
+      <c r="B46" t="s">
         <v>290</v>
-      </c>
-      <c r="B46" t="s">
-        <v>291</v>
       </c>
     </row>
     <row r="47" spans="1:2">
       <c r="A47" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B47" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="48" spans="1:2">
       <c r="A48" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B48" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="49" spans="1:2">
       <c r="A49" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B49" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="50" spans="1:2">
       <c r="A50" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B50" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="51" spans="1:2">
       <c r="A51" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="B51" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
     </row>
     <row r="52" spans="1:2">
       <c r="A52" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B52" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="53" spans="1:2">
       <c r="A53" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B53" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="54" spans="1:2">
       <c r="A54" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B54" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="55" spans="1:2">
       <c r="A55" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B55" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="56" spans="1:2">
       <c r="A56" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B56" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="57" spans="1:2">
       <c r="A57" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B57" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="58" spans="1:2">
       <c r="A58" t="s">
+        <v>180</v>
+      </c>
+      <c r="B58" t="s">
         <v>181</v>
-      </c>
-      <c r="B58" t="s">
-        <v>182</v>
       </c>
     </row>
     <row r="59" spans="1:2">
       <c r="A59" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B59" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="60" spans="1:2">
       <c r="A60" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B60" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="61" spans="1:2">
       <c r="A61" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B61" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="62" spans="1:2">
       <c r="A62" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B62" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="63" spans="1:2">
       <c r="A63" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B63" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="64" spans="1:2">
       <c r="A64" t="s">
+        <v>193</v>
+      </c>
+      <c r="B64" t="s">
         <v>194</v>
-      </c>
-      <c r="B64" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="65" spans="1:2">
       <c r="A65" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B65" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="66" spans="1:2">
       <c r="A66" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B66" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="67" spans="1:2">
       <c r="A67" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B67" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="68" spans="1:2">
       <c r="A68" t="s">
+        <v>198</v>
+      </c>
+      <c r="B68" t="s">
         <v>199</v>
-      </c>
-      <c r="B68" t="s">
-        <v>200</v>
       </c>
     </row>
     <row r="69" spans="1:2">
       <c r="A69" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B69" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="70" spans="1:2">
       <c r="A70" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B70" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="71" spans="1:2">
       <c r="A71" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B71" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="72" spans="1:2">
       <c r="A72" t="s">
+        <v>283</v>
+      </c>
+      <c r="B72" t="s">
         <v>284</v>
-      </c>
-      <c r="B72" t="s">
-        <v>285</v>
       </c>
     </row>
     <row r="73" spans="1:2">
       <c r="A73" t="s">
+        <v>209</v>
+      </c>
+      <c r="B73" t="s">
         <v>210</v>
-      </c>
-      <c r="B73" t="s">
-        <v>211</v>
       </c>
     </row>
     <row r="74" spans="1:2">
       <c r="A74" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B74" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="75" spans="1:2">
       <c r="A75" t="s">
+        <v>212</v>
+      </c>
+      <c r="B75" t="s">
         <v>213</v>
-      </c>
-      <c r="B75" t="s">
-        <v>214</v>
       </c>
     </row>
     <row r="76" spans="1:2">
       <c r="A76" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B76" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="77" spans="1:2">
       <c r="A77" t="s">
+        <v>217</v>
+      </c>
+      <c r="B77" t="s">
         <v>218</v>
-      </c>
-      <c r="B77" t="s">
-        <v>219</v>
       </c>
     </row>
     <row r="78" spans="1:2">
       <c r="A78" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B78" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="79" spans="1:2">
       <c r="A79" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B79" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="80" spans="1:2">
       <c r="A80" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B80" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
     </row>
     <row r="81" spans="1:2">
       <c r="A81" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B81" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="82" spans="1:2">
       <c r="A82" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B82" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="83" spans="1:2">
       <c r="A83" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B83" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="84" spans="1:2">
       <c r="A84" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B84" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="85" spans="1:2">
       <c r="A85" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="B85" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="86" spans="1:2">
       <c r="A86" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="B86" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
     </row>
     <row r="87" spans="1:2">
       <c r="A87" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="B87" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
     </row>
     <row r="88" spans="1:2">
       <c r="A88" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="B88" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
     </row>
     <row r="89" spans="1:2">
       <c r="A89" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B89" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
     </row>
     <row r="90" spans="1:2">
       <c r="A90" t="s">
+        <v>356</v>
+      </c>
+      <c r="B90" t="s">
         <v>358</v>
-      </c>
-      <c r="B90" t="s">
-        <v>360</v>
       </c>
     </row>
     <row r="91" spans="1:2">
       <c r="A91" t="s">
+        <v>357</v>
+      </c>
+      <c r="B91" t="s">
         <v>359</v>
-      </c>
-      <c r="B91" t="s">
-        <v>361</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added Main.xaml level arguement to bypass trigger email Modified the selectors for the Process Monitor status validation
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27126"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\57841C\Documents\UiPath\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\svc_prod.robot01\Documents\UiPath\P002_090_PayCyleAfternoon_Dispatcher\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABF3CEC1-98C4-4B64-A8B9-DC61FD47D28A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32C4BCCB-1F4E-4FEC-B2B3-8AAC500D11DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -997,9 +997,6 @@
     <t>\d+\s-\s\w+\sno success</t>
   </si>
   <si>
-    <t>00:04:00</t>
-  </si>
-  <si>
     <t>PeopleSoftLoginCredentailsFolderName</t>
   </si>
   <si>
@@ -1220,6 +1217,9 @@
   </si>
   <si>
     <t>PROD</t>
+  </si>
+  <si>
+    <t>00:00:10</t>
   </si>
 </sst>
 </file>
@@ -1577,9 +1577,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1617,7 +1617,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1723,7 +1723,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1865,7 +1865,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1963,7 +1963,7 @@
     </row>
     <row r="6" spans="1:26">
       <c r="A6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="B6" t="str">
         <f>_xlfn.CONCAT(Constants!$B$18,"/P002_090_PayCycleAfternoon")</f>
@@ -1975,7 +1975,7 @@
         <v>48</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="C7" t="s">
         <v>49</v>
@@ -1986,7 +1986,7 @@
         <v>50</v>
       </c>
       <c r="B8" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="C8" t="s">
         <v>51</v>
@@ -2052,7 +2052,7 @@
         <v>64</v>
       </c>
       <c r="B14" s="21" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="C14" s="5" t="s">
         <v>65</v>
@@ -2063,7 +2063,7 @@
         <v>66</v>
       </c>
       <c r="B15" s="21" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="C15" s="5" t="s">
         <v>67</v>
@@ -2074,7 +2074,7 @@
         <v>68</v>
       </c>
       <c r="B16" s="22" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="C16" s="5" t="s">
         <v>69</v>
@@ -2236,7 +2236,7 @@
         <v>148</v>
       </c>
       <c r="B34" s="11" t="s">
-        <v>319</v>
+        <v>393</v>
       </c>
     </row>
     <row r="35" spans="1:2">
@@ -2252,7 +2252,7 @@
         <v>215</v>
       </c>
       <c r="B36">
-        <v>5</v>
+        <v>120</v>
       </c>
     </row>
     <row r="37" spans="1:2">
@@ -2276,7 +2276,7 @@
         <v>234</v>
       </c>
       <c r="B39" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="40" spans="1:2">
@@ -2369,7 +2369,7 @@
     </row>
     <row r="51" spans="1:2">
       <c r="A51" s="19" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="B51" t="s">
         <v>311</v>
@@ -2377,7 +2377,7 @@
     </row>
     <row r="52" spans="1:2" ht="43.5">
       <c r="A52" s="19" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="B52" s="3" t="s">
         <v>312</v>
@@ -2385,18 +2385,18 @@
     </row>
     <row r="53" spans="1:2">
       <c r="A53" s="24" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="B53" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="54" spans="1:2" ht="43.5">
       <c r="A54" s="24" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -2484,10 +2484,10 @@
     </row>
     <row r="66" spans="1:2">
       <c r="A66" t="s">
+        <v>364</v>
+      </c>
+      <c r="B66" t="s">
         <v>365</v>
-      </c>
-      <c r="B66" t="s">
-        <v>366</v>
       </c>
     </row>
   </sheetData>
@@ -2676,10 +2676,10 @@
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="B18" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
     </row>
   </sheetData>
@@ -2747,7 +2747,7 @@
         <v>PROD/P002_090_PayCycleAfternoon</v>
       </c>
       <c r="D2" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
     </row>
     <row r="3" spans="1:26">
@@ -2755,7 +2755,7 @@
         <v>41</v>
       </c>
       <c r="B3" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="C3" t="str">
         <f>_xlfn.CONCAT(Constants!$B$18,"/P002_090_PayCycleAfternoon")</f>
@@ -2764,10 +2764,10 @@
     </row>
     <row r="4" spans="1:26">
       <c r="A4" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="B4" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C4" t="str">
         <f>_xlfn.CONCAT(Constants!$B$18,"/P002_090_PayCycleAfternoon")</f>
@@ -2779,7 +2779,7 @@
         <v>44</v>
       </c>
       <c r="B5" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C5" t="str">
         <f>_xlfn.CONCAT(Constants!$B$18,"/P002_090_PayCycleAfternoon")</f>
@@ -2791,7 +2791,7 @@
         <v>45</v>
       </c>
       <c r="B6" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="C6" t="str">
         <f>_xlfn.CONCAT(Constants!$B$18,"/P002_090_PayCycleAfternoon")</f>
@@ -2803,7 +2803,7 @@
         <v>46</v>
       </c>
       <c r="B7" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="C7" t="str">
         <f>_xlfn.CONCAT(Constants!$B$18,"/P002_090_PayCycleAfternoon")</f>
@@ -2815,7 +2815,7 @@
         <v>47</v>
       </c>
       <c r="B8" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="C8" t="str">
         <f>_xlfn.CONCAT(Constants!$B$18,"/P002_090_PayCycleAfternoon")</f>
@@ -2827,7 +2827,7 @@
         <v>123</v>
       </c>
       <c r="B9" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C9" t="str">
         <f>_xlfn.CONCAT(Constants!$B$18,"/P002_090_PayCycleAfternoon")</f>
@@ -2839,7 +2839,7 @@
         <v>295</v>
       </c>
       <c r="B10" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="C10" t="str">
         <f>_xlfn.CONCAT(Constants!$B$18,"/P002_090_PayCycleAfternoon")</f>
@@ -2851,7 +2851,7 @@
         <v>240</v>
       </c>
       <c r="B11" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="C11" t="str">
         <f>_xlfn.CONCAT(Constants!$B$18,"/P002_090_PayCycleAfternoon")</f>
@@ -2863,7 +2863,7 @@
         <v>241</v>
       </c>
       <c r="B12" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="C12" t="str">
         <f>_xlfn.CONCAT(Constants!$B$18,"/P002_090_PayCycleAfternoon")</f>
@@ -2875,7 +2875,7 @@
         <v>244</v>
       </c>
       <c r="B13" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="C13" t="str">
         <f>_xlfn.CONCAT(Constants!$B$18,"/P002_090_PayCycleAfternoon")</f>
@@ -2887,7 +2887,7 @@
         <v>245</v>
       </c>
       <c r="B14" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C14" t="str">
         <f>_xlfn.CONCAT(Constants!$B$18,"/P002_090_PayCycleAfternoon")</f>
@@ -2899,7 +2899,7 @@
         <v>257</v>
       </c>
       <c r="B15" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="C15" t="str">
         <f>_xlfn.CONCAT(Constants!$B$18,"/P002_090_PayCycleAfternoon")</f>
@@ -2911,7 +2911,7 @@
         <v>258</v>
       </c>
       <c r="B16" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="C16" t="str">
         <f>_xlfn.CONCAT(Constants!$B$18,"/P002_090_PayCycleAfternoon")</f>
@@ -2923,7 +2923,7 @@
         <v>253</v>
       </c>
       <c r="B17" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="C17" t="str">
         <f>_xlfn.CONCAT(Constants!$B$18,"/P002_090_PayCycleAfternoon")</f>
@@ -2935,7 +2935,7 @@
         <v>254</v>
       </c>
       <c r="B18" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="C18" t="str">
         <f>_xlfn.CONCAT(Constants!$B$18,"/P002_090_PayCycleAfternoon")</f>
@@ -2947,7 +2947,7 @@
         <v>316</v>
       </c>
       <c r="B19" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="C19" t="str">
         <f>_xlfn.CONCAT(Constants!$B$18,"/P002_090_PayCycleAfternoon")</f>
@@ -2959,7 +2959,7 @@
         <v>317</v>
       </c>
       <c r="B20" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="C20" t="str">
         <f>_xlfn.CONCAT(Constants!$B$18,"/P002_090_PayCycleAfternoon")</f>
@@ -2968,10 +2968,10 @@
     </row>
     <row r="21" spans="1:3">
       <c r="A21" s="19" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="B21" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="C21" t="str">
         <f>_xlfn.CONCAT(Constants!$B$18,"/P002_090_PayCycleAfternoon")</f>
@@ -2980,10 +2980,10 @@
     </row>
     <row r="22" spans="1:3">
       <c r="A22" s="19" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="B22" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="C22" t="str">
         <f>_xlfn.CONCAT(Constants!$B$18,"/P002_090_PayCycleAfternoon")</f>
@@ -2992,10 +2992,10 @@
     </row>
     <row r="23" spans="1:3">
       <c r="A23" s="24" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="B23" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="C23" t="str">
         <f>_xlfn.CONCAT(Constants!$B$18,"/P002_090_PayCycleAfternoon")</f>
@@ -3004,10 +3004,10 @@
     </row>
     <row r="24" spans="1:3">
       <c r="A24" s="24" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="B24" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="C24" t="str">
         <f>_xlfn.CONCAT(Constants!$B$18,"/P002_090_PayCycleAfternoon")</f>
@@ -3016,10 +3016,10 @@
     </row>
     <row r="25" spans="1:3">
       <c r="A25" s="19" t="s">
+        <v>351</v>
+      </c>
+      <c r="B25" t="s">
         <v>352</v>
-      </c>
-      <c r="B25" t="s">
-        <v>353</v>
       </c>
       <c r="C25" t="str">
         <f>_xlfn.CONCAT(Constants!$B$18,"/P002_090_PayCycleAfternoon")</f>
@@ -3142,18 +3142,18 @@
     </row>
     <row r="10" spans="1:26">
       <c r="A10" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="B10" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="11" spans="1:26">
       <c r="A11" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="B11" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
     </row>
     <row r="12" spans="1:26">
@@ -3174,18 +3174,18 @@
     </row>
     <row r="14" spans="1:26">
       <c r="A14" t="s">
+        <v>375</v>
+      </c>
+      <c r="B14" t="s">
         <v>376</v>
-      </c>
-      <c r="B14" t="s">
-        <v>377</v>
       </c>
     </row>
     <row r="15" spans="1:26">
       <c r="A15" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="B15" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="16" spans="1:26">
@@ -3326,26 +3326,26 @@
     </row>
     <row r="33" spans="1:2">
       <c r="A33" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="B33" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="34" spans="1:2">
       <c r="A34" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B34" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="35" spans="1:2">
       <c r="A35" t="s">
+        <v>372</v>
+      </c>
+      <c r="B35" t="s">
         <v>373</v>
-      </c>
-      <c r="B35" t="s">
-        <v>374</v>
       </c>
     </row>
     <row r="36" spans="1:2">
@@ -3470,10 +3470,10 @@
     </row>
     <row r="51" spans="1:2">
       <c r="A51" t="s">
+        <v>349</v>
+      </c>
+      <c r="B51" t="s">
         <v>350</v>
-      </c>
-      <c r="B51" t="s">
-        <v>351</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -3705,7 +3705,7 @@
         <v>206</v>
       </c>
       <c r="B80" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -3750,50 +3750,50 @@
     </row>
     <row r="86" spans="1:2">
       <c r="A86" t="s">
+        <v>353</v>
+      </c>
+      <c r="B86" t="s">
         <v>354</v>
-      </c>
-      <c r="B86" t="s">
-        <v>355</v>
       </c>
     </row>
     <row r="87" spans="1:2">
       <c r="A87" t="s">
+        <v>359</v>
+      </c>
+      <c r="B87" t="s">
         <v>360</v>
-      </c>
-      <c r="B87" t="s">
-        <v>361</v>
       </c>
     </row>
     <row r="88" spans="1:2">
       <c r="A88" t="s">
+        <v>361</v>
+      </c>
+      <c r="B88" t="s">
         <v>362</v>
-      </c>
-      <c r="B88" t="s">
-        <v>363</v>
       </c>
     </row>
     <row r="89" spans="1:2">
       <c r="A89" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B89" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
     </row>
     <row r="90" spans="1:2">
       <c r="A90" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="B90" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
     </row>
     <row r="91" spans="1:2">
       <c r="A91" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="B91" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updates to Process Monitor entry package
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\svc_prod.robot01\Documents\UiPath\P002_090_PayCyleAfternoon_Dispatcher\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32C4BCCB-1F4E-4FEC-B2B3-8AAC500D11DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22ADBF87-9091-495A-A7FA-DE9093EAD265}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="406" uniqueCount="394">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="410" uniqueCount="398">
   <si>
     <t>Name</t>
   </si>
@@ -1220,6 +1220,18 @@
   </si>
   <si>
     <t>00:00:10</t>
+  </si>
+  <si>
+    <t>UserIDNotFoundSE</t>
+  </si>
+  <si>
+    <t>ProcessNameNotFoundSE</t>
+  </si>
+  <si>
+    <t>The bot could not validate that the selected Process Name was entered into the Process Monitor window.</t>
+  </si>
+  <si>
+    <t>The bot could not validate that the selected Process Monitor UserID has been entered.</t>
   </si>
 </sst>
 </file>
@@ -3034,7 +3046,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C1D9DC59-3960-42CB-B3EC-EFF452A90D4F}">
-  <dimension ref="A1:Z91"/>
+  <dimension ref="A1:Z93"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="41.08984375" bestFit="1" customWidth="1"/>
@@ -3078,490 +3090,490 @@
     </row>
     <row r="2" spans="1:26">
       <c r="A2" t="s">
-        <v>92</v>
+        <v>176</v>
       </c>
       <c r="B2" t="s">
-        <v>93</v>
+        <v>187</v>
       </c>
     </row>
     <row r="3" spans="1:26">
       <c r="A3" t="s">
-        <v>281</v>
+        <v>174</v>
       </c>
       <c r="B3" t="s">
-        <v>282</v>
+        <v>185</v>
       </c>
     </row>
     <row r="4" spans="1:26">
       <c r="A4" t="s">
-        <v>280</v>
+        <v>175</v>
       </c>
       <c r="B4" t="s">
-        <v>232</v>
+        <v>186</v>
       </c>
     </row>
     <row r="5" spans="1:26">
       <c r="A5" t="s">
-        <v>94</v>
+        <v>173</v>
       </c>
       <c r="B5" t="s">
-        <v>95</v>
+        <v>177</v>
       </c>
     </row>
     <row r="6" spans="1:26">
       <c r="A6" t="s">
-        <v>96</v>
+        <v>283</v>
       </c>
       <c r="B6" t="s">
-        <v>97</v>
+        <v>284</v>
       </c>
     </row>
     <row r="7" spans="1:26">
       <c r="A7" t="s">
-        <v>98</v>
+        <v>220</v>
       </c>
       <c r="B7" t="s">
-        <v>99</v>
+        <v>219</v>
       </c>
     </row>
     <row r="8" spans="1:26">
       <c r="A8" t="s">
-        <v>102</v>
+        <v>221</v>
       </c>
       <c r="B8" t="s">
-        <v>101</v>
+        <v>219</v>
       </c>
     </row>
     <row r="9" spans="1:26">
       <c r="A9" t="s">
-        <v>105</v>
+        <v>214</v>
       </c>
       <c r="B9" t="s">
-        <v>106</v>
+        <v>216</v>
       </c>
     </row>
     <row r="10" spans="1:26">
       <c r="A10" t="s">
-        <v>346</v>
+        <v>217</v>
       </c>
       <c r="B10" t="s">
-        <v>345</v>
+        <v>218</v>
       </c>
     </row>
     <row r="11" spans="1:26">
       <c r="A11" t="s">
-        <v>348</v>
+        <v>161</v>
       </c>
       <c r="B11" t="s">
-        <v>347</v>
+        <v>163</v>
       </c>
     </row>
     <row r="12" spans="1:26">
       <c r="A12" t="s">
-        <v>296</v>
+        <v>144</v>
       </c>
       <c r="B12" t="s">
-        <v>299</v>
+        <v>172</v>
       </c>
     </row>
     <row r="13" spans="1:26">
       <c r="A13" t="s">
-        <v>297</v>
+        <v>142</v>
       </c>
       <c r="B13" t="s">
-        <v>298</v>
+        <v>169</v>
       </c>
     </row>
     <row r="14" spans="1:26">
       <c r="A14" t="s">
-        <v>375</v>
+        <v>143</v>
       </c>
       <c r="B14" t="s">
-        <v>376</v>
+        <v>171</v>
       </c>
     </row>
     <row r="15" spans="1:26">
       <c r="A15" t="s">
-        <v>378</v>
+        <v>141</v>
       </c>
       <c r="B15" t="s">
-        <v>377</v>
+        <v>140</v>
       </c>
     </row>
     <row r="16" spans="1:26">
       <c r="A16" t="s">
-        <v>309</v>
+        <v>133</v>
       </c>
       <c r="B16" t="s">
-        <v>308</v>
+        <v>139</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" t="s">
-        <v>103</v>
+        <v>131</v>
       </c>
       <c r="B17" t="s">
-        <v>107</v>
+        <v>137</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" t="s">
-        <v>104</v>
+        <v>132</v>
       </c>
       <c r="B18" t="s">
-        <v>108</v>
+        <v>138</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" t="s">
-        <v>110</v>
+        <v>130</v>
       </c>
       <c r="B19" t="s">
-        <v>113</v>
+        <v>136</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" t="s">
-        <v>301</v>
+        <v>355</v>
       </c>
       <c r="B20" t="s">
-        <v>300</v>
+        <v>357</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21" t="s">
-        <v>111</v>
+        <v>356</v>
       </c>
       <c r="B21" t="s">
-        <v>114</v>
+        <v>358</v>
       </c>
     </row>
     <row r="22" spans="1:2">
       <c r="A22" t="s">
-        <v>112</v>
+        <v>353</v>
       </c>
       <c r="B22" t="s">
-        <v>115</v>
+        <v>354</v>
       </c>
     </row>
     <row r="23" spans="1:2">
       <c r="A23" t="s">
-        <v>116</v>
+        <v>149</v>
       </c>
       <c r="B23" t="s">
-        <v>119</v>
+        <v>150</v>
       </c>
     </row>
     <row r="24" spans="1:2">
       <c r="A24" t="s">
-        <v>302</v>
+        <v>261</v>
       </c>
       <c r="B24" t="s">
-        <v>303</v>
+        <v>264</v>
       </c>
     </row>
     <row r="25" spans="1:2">
       <c r="A25" t="s">
-        <v>117</v>
+        <v>262</v>
       </c>
       <c r="B25" t="s">
-        <v>120</v>
+        <v>265</v>
       </c>
     </row>
     <row r="26" spans="1:2">
       <c r="A26" t="s">
-        <v>118</v>
+        <v>260</v>
       </c>
       <c r="B26" t="s">
-        <v>121</v>
+        <v>263</v>
       </c>
     </row>
     <row r="27" spans="1:2">
       <c r="A27" t="s">
-        <v>130</v>
+        <v>361</v>
       </c>
       <c r="B27" t="s">
-        <v>136</v>
+        <v>362</v>
       </c>
     </row>
     <row r="28" spans="1:2">
       <c r="A28" t="s">
-        <v>246</v>
+        <v>363</v>
       </c>
       <c r="B28" t="s">
-        <v>248</v>
+        <v>362</v>
       </c>
     </row>
     <row r="29" spans="1:2">
       <c r="A29" t="s">
-        <v>247</v>
+        <v>359</v>
       </c>
       <c r="B29" t="s">
-        <v>248</v>
+        <v>360</v>
       </c>
     </row>
     <row r="30" spans="1:2">
       <c r="A30" t="s">
-        <v>135</v>
+        <v>309</v>
       </c>
       <c r="B30" t="s">
-        <v>134</v>
+        <v>308</v>
       </c>
     </row>
     <row r="31" spans="1:2">
       <c r="A31" t="s">
-        <v>292</v>
+        <v>209</v>
       </c>
       <c r="B31" t="s">
-        <v>293</v>
+        <v>210</v>
       </c>
     </row>
     <row r="32" spans="1:2">
       <c r="A32" t="s">
-        <v>266</v>
+        <v>211</v>
       </c>
       <c r="B32" t="s">
-        <v>294</v>
+        <v>210</v>
       </c>
     </row>
     <row r="33" spans="1:2">
       <c r="A33" t="s">
-        <v>370</v>
+        <v>111</v>
       </c>
       <c r="B33" t="s">
-        <v>374</v>
+        <v>114</v>
       </c>
     </row>
     <row r="34" spans="1:2">
       <c r="A34" t="s">
-        <v>371</v>
+        <v>112</v>
       </c>
       <c r="B34" t="s">
-        <v>374</v>
+        <v>115</v>
       </c>
     </row>
     <row r="35" spans="1:2">
       <c r="A35" t="s">
-        <v>372</v>
+        <v>110</v>
       </c>
       <c r="B35" t="s">
-        <v>373</v>
+        <v>113</v>
       </c>
     </row>
     <row r="36" spans="1:2">
       <c r="A36" t="s">
-        <v>131</v>
+        <v>301</v>
       </c>
       <c r="B36" t="s">
-        <v>137</v>
+        <v>300</v>
       </c>
     </row>
     <row r="37" spans="1:2">
       <c r="A37" t="s">
-        <v>132</v>
+        <v>212</v>
       </c>
       <c r="B37" t="s">
-        <v>138</v>
+        <v>213</v>
       </c>
     </row>
     <row r="38" spans="1:2">
       <c r="A38" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B38" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
     </row>
     <row r="39" spans="1:2">
       <c r="A39" t="s">
-        <v>141</v>
+        <v>292</v>
       </c>
       <c r="B39" t="s">
-        <v>140</v>
+        <v>293</v>
       </c>
     </row>
     <row r="40" spans="1:2">
       <c r="A40" t="s">
-        <v>154</v>
+        <v>179</v>
       </c>
       <c r="B40" t="s">
-        <v>152</v>
+        <v>178</v>
       </c>
     </row>
     <row r="41" spans="1:2">
       <c r="A41" t="s">
-        <v>153</v>
+        <v>180</v>
       </c>
       <c r="B41" t="s">
-        <v>151</v>
+        <v>181</v>
       </c>
     </row>
     <row r="42" spans="1:2">
       <c r="A42" t="s">
-        <v>149</v>
+        <v>289</v>
       </c>
       <c r="B42" t="s">
-        <v>150</v>
+        <v>290</v>
       </c>
     </row>
     <row r="43" spans="1:2">
       <c r="A43" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B43" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="44" spans="1:2">
       <c r="A44" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B44" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="45" spans="1:2">
       <c r="A45" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B45" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
     </row>
     <row r="46" spans="1:2">
       <c r="A46" t="s">
-        <v>289</v>
+        <v>170</v>
       </c>
       <c r="B46" t="s">
-        <v>290</v>
+        <v>313</v>
       </c>
     </row>
     <row r="47" spans="1:2">
       <c r="A47" t="s">
-        <v>161</v>
+        <v>349</v>
       </c>
       <c r="B47" t="s">
-        <v>163</v>
+        <v>350</v>
       </c>
     </row>
     <row r="48" spans="1:2">
       <c r="A48" t="s">
-        <v>162</v>
+        <v>250</v>
       </c>
       <c r="B48" t="s">
-        <v>164</v>
+        <v>249</v>
       </c>
     </row>
     <row r="49" spans="1:2">
       <c r="A49" t="s">
-        <v>168</v>
+        <v>193</v>
       </c>
       <c r="B49" t="s">
-        <v>167</v>
+        <v>194</v>
       </c>
     </row>
     <row r="50" spans="1:2">
       <c r="A50" t="s">
-        <v>170</v>
+        <v>196</v>
       </c>
       <c r="B50" t="s">
-        <v>313</v>
+        <v>195</v>
       </c>
     </row>
     <row r="51" spans="1:2">
       <c r="A51" t="s">
-        <v>349</v>
+        <v>375</v>
       </c>
       <c r="B51" t="s">
-        <v>350</v>
+        <v>376</v>
       </c>
     </row>
     <row r="52" spans="1:2">
       <c r="A52" t="s">
-        <v>250</v>
+        <v>378</v>
       </c>
       <c r="B52" t="s">
-        <v>249</v>
+        <v>377</v>
       </c>
     </row>
     <row r="53" spans="1:2">
       <c r="A53" t="s">
-        <v>142</v>
+        <v>346</v>
       </c>
       <c r="B53" t="s">
-        <v>169</v>
+        <v>345</v>
       </c>
     </row>
     <row r="54" spans="1:2">
       <c r="A54" t="s">
-        <v>143</v>
+        <v>105</v>
       </c>
       <c r="B54" t="s">
-        <v>171</v>
+        <v>106</v>
       </c>
     </row>
     <row r="55" spans="1:2">
       <c r="A55" t="s">
-        <v>144</v>
+        <v>296</v>
       </c>
       <c r="B55" t="s">
-        <v>172</v>
+        <v>299</v>
       </c>
     </row>
     <row r="56" spans="1:2">
       <c r="A56" t="s">
-        <v>173</v>
+        <v>348</v>
       </c>
       <c r="B56" t="s">
-        <v>177</v>
+        <v>347</v>
       </c>
     </row>
     <row r="57" spans="1:2">
       <c r="A57" t="s">
-        <v>179</v>
+        <v>297</v>
       </c>
       <c r="B57" t="s">
-        <v>178</v>
+        <v>298</v>
       </c>
     </row>
     <row r="58" spans="1:2">
       <c r="A58" t="s">
-        <v>180</v>
+        <v>103</v>
       </c>
       <c r="B58" t="s">
-        <v>181</v>
+        <v>107</v>
       </c>
     </row>
     <row r="59" spans="1:2">
       <c r="A59" t="s">
-        <v>183</v>
+        <v>104</v>
       </c>
       <c r="B59" t="s">
-        <v>182</v>
+        <v>108</v>
       </c>
     </row>
     <row r="60" spans="1:2">
       <c r="A60" t="s">
-        <v>174</v>
+        <v>102</v>
       </c>
       <c r="B60" t="s">
-        <v>185</v>
+        <v>101</v>
       </c>
     </row>
     <row r="61" spans="1:2">
       <c r="A61" t="s">
-        <v>175</v>
+        <v>190</v>
       </c>
       <c r="B61" t="s">
-        <v>186</v>
+        <v>192</v>
       </c>
     </row>
     <row r="62" spans="1:2">
       <c r="A62" t="s">
-        <v>176</v>
+        <v>191</v>
       </c>
       <c r="B62" t="s">
-        <v>187</v>
+        <v>197</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -3574,229 +3586,248 @@
     </row>
     <row r="64" spans="1:2">
       <c r="A64" t="s">
-        <v>193</v>
+        <v>154</v>
       </c>
       <c r="B64" t="s">
-        <v>194</v>
+        <v>152</v>
       </c>
     </row>
     <row r="65" spans="1:2">
       <c r="A65" t="s">
-        <v>196</v>
+        <v>153</v>
       </c>
       <c r="B65" t="s">
-        <v>195</v>
+        <v>151</v>
       </c>
     </row>
     <row r="66" spans="1:2">
       <c r="A66" t="s">
-        <v>190</v>
+        <v>156</v>
       </c>
       <c r="B66" t="s">
-        <v>192</v>
+        <v>155</v>
       </c>
     </row>
     <row r="67" spans="1:2">
       <c r="A67" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
       <c r="B67" t="s">
-        <v>197</v>
+        <v>182</v>
       </c>
     </row>
     <row r="68" spans="1:2">
       <c r="A68" t="s">
-        <v>198</v>
+        <v>302</v>
       </c>
       <c r="B68" t="s">
-        <v>199</v>
+        <v>303</v>
       </c>
     </row>
     <row r="69" spans="1:2">
       <c r="A69" t="s">
-        <v>200</v>
+        <v>168</v>
       </c>
       <c r="B69" t="s">
-        <v>202</v>
+        <v>167</v>
       </c>
     </row>
     <row r="70" spans="1:2">
       <c r="A70" t="s">
-        <v>201</v>
+        <v>266</v>
       </c>
       <c r="B70" t="s">
-        <v>203</v>
+        <v>294</v>
       </c>
     </row>
     <row r="71" spans="1:2">
       <c r="A71" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B71" t="s">
-        <v>204</v>
+        <v>223</v>
       </c>
     </row>
     <row r="72" spans="1:2">
       <c r="A72" t="s">
-        <v>283</v>
+        <v>206</v>
       </c>
       <c r="B72" t="s">
-        <v>284</v>
+        <v>380</v>
       </c>
     </row>
     <row r="73" spans="1:2">
       <c r="A73" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B73" t="s">
-        <v>210</v>
+        <v>222</v>
       </c>
     </row>
     <row r="74" spans="1:2">
       <c r="A74" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
       <c r="B74" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
     </row>
     <row r="75" spans="1:2">
       <c r="A75" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
       <c r="B75" t="s">
-        <v>213</v>
+        <v>202</v>
       </c>
     </row>
     <row r="76" spans="1:2">
       <c r="A76" t="s">
-        <v>214</v>
+        <v>201</v>
       </c>
       <c r="B76" t="s">
-        <v>216</v>
+        <v>203</v>
       </c>
     </row>
     <row r="77" spans="1:2">
       <c r="A77" t="s">
-        <v>217</v>
+        <v>198</v>
       </c>
       <c r="B77" t="s">
-        <v>218</v>
+        <v>199</v>
       </c>
     </row>
     <row r="78" spans="1:2">
       <c r="A78" t="s">
-        <v>220</v>
+        <v>372</v>
       </c>
       <c r="B78" t="s">
-        <v>219</v>
+        <v>373</v>
       </c>
     </row>
     <row r="79" spans="1:2">
       <c r="A79" t="s">
-        <v>221</v>
+        <v>246</v>
       </c>
       <c r="B79" t="s">
-        <v>219</v>
+        <v>248</v>
       </c>
     </row>
     <row r="80" spans="1:2">
       <c r="A80" t="s">
-        <v>206</v>
+        <v>247</v>
       </c>
       <c r="B80" t="s">
-        <v>380</v>
+        <v>248</v>
       </c>
     </row>
     <row r="81" spans="1:2">
       <c r="A81" t="s">
-        <v>207</v>
+        <v>370</v>
       </c>
       <c r="B81" t="s">
-        <v>223</v>
+        <v>374</v>
       </c>
     </row>
     <row r="82" spans="1:2">
       <c r="A82" t="s">
-        <v>208</v>
+        <v>371</v>
       </c>
       <c r="B82" t="s">
-        <v>222</v>
+        <v>374</v>
       </c>
     </row>
     <row r="83" spans="1:2">
       <c r="A83" t="s">
-        <v>260</v>
+        <v>281</v>
       </c>
       <c r="B83" t="s">
-        <v>263</v>
+        <v>282</v>
       </c>
     </row>
     <row r="84" spans="1:2">
       <c r="A84" t="s">
-        <v>261</v>
+        <v>280</v>
       </c>
       <c r="B84" t="s">
-        <v>264</v>
+        <v>232</v>
       </c>
     </row>
     <row r="85" spans="1:2">
       <c r="A85" t="s">
-        <v>262</v>
+        <v>98</v>
       </c>
       <c r="B85" t="s">
-        <v>265</v>
+        <v>99</v>
       </c>
     </row>
     <row r="86" spans="1:2">
       <c r="A86" t="s">
-        <v>353</v>
+        <v>94</v>
       </c>
       <c r="B86" t="s">
-        <v>354</v>
+        <v>95</v>
       </c>
     </row>
     <row r="87" spans="1:2">
       <c r="A87" t="s">
-        <v>359</v>
+        <v>96</v>
       </c>
       <c r="B87" t="s">
-        <v>360</v>
+        <v>97</v>
       </c>
     </row>
     <row r="88" spans="1:2">
       <c r="A88" t="s">
-        <v>361</v>
+        <v>92</v>
       </c>
       <c r="B88" t="s">
-        <v>362</v>
+        <v>93</v>
       </c>
     </row>
     <row r="89" spans="1:2">
       <c r="A89" t="s">
-        <v>363</v>
+        <v>117</v>
       </c>
       <c r="B89" t="s">
-        <v>362</v>
+        <v>120</v>
       </c>
     </row>
     <row r="90" spans="1:2">
       <c r="A90" t="s">
-        <v>355</v>
+        <v>118</v>
       </c>
       <c r="B90" t="s">
-        <v>357</v>
+        <v>121</v>
       </c>
     </row>
     <row r="91" spans="1:2">
       <c r="A91" t="s">
-        <v>356</v>
+        <v>116</v>
       </c>
       <c r="B91" t="s">
-        <v>358</v>
+        <v>119</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2">
+      <c r="A92" t="s">
+        <v>394</v>
+      </c>
+      <c r="B92" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2">
+      <c r="A93" t="s">
+        <v>395</v>
+      </c>
+      <c r="B93" t="s">
+        <v>396</v>
       </c>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C91">
+    <sortCondition ref="A2:A91"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>